<commit_message>
Add voyage SWAL 2609N BKK02 (66 containers, storage 14,600); LCH01 re-run with LOAD2
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VOYAGES/2026-10-23_KST_SWAL_2609N_THLCH_LCH01/2026-10-23_KST_SWAL_2609N_THLCH_LCH01.xlsx
+++ b/VOYAGES/2026-10-23_KST_SWAL_2609N_THLCH_LCH01/2026-10-23_KST_SWAL_2609N_THLCH_LCH01.xlsx
@@ -995,14 +995,14 @@
     <row r="25">
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>ไฟล์ต้นฉบับ: 10-23-BKG.xls, 10-23-GATE.xls, 10-23-LOAD.xls</t>
+          <t>ไฟล์ต้นฉบับ: 10-23-BKG.xls, 10-23-GATE2.xls, 10-23-LOAD2.xls</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>คำนวณเมื่อ: 23/10/2026 11:15</t>
+          <t>คำนวณเมื่อ: 23/10/2026 11:20</t>
         </is>
       </c>
     </row>
@@ -9729,7 +9729,7 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>SKLU1586238</t>
+          <t>SKLU2101727</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="AA15" s="12" t="n">
-        <v>12490</v>
+        <v>23780</v>
       </c>
       <c r="AB15" s="12" t="inlineStr">
         <is>
@@ -9870,7 +9870,7 @@
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>SKLU2101727</t>
+          <t>SKLU1553830</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -9995,7 +9995,7 @@
         </is>
       </c>
       <c r="AA16" s="12" t="n">
-        <v>23780</v>
+        <v>24290</v>
       </c>
       <c r="AB16" s="12" t="inlineStr">
         <is>
@@ -10011,7 +10011,7 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>SKLU2105770</t>
+          <t>SKLU1586238</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="X17" s="12" t="inlineStr">
         <is>
-          <t>VFD</t>
+          <t>VED</t>
         </is>
       </c>
       <c r="Y17" s="12" t="inlineStr">
@@ -10136,7 +10136,7 @@
         </is>
       </c>
       <c r="AA17" s="12" t="n">
-        <v>23200</v>
+        <v>12490</v>
       </c>
       <c r="AB17" s="12" t="inlineStr">
         <is>
@@ -10293,7 +10293,7 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>SKLU1553830</t>
+          <t>SKLU2105770</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -10404,7 +10404,7 @@
       </c>
       <c r="X19" s="12" t="inlineStr">
         <is>
-          <t>VED</t>
+          <t>VFD</t>
         </is>
       </c>
       <c r="Y19" s="12" t="inlineStr">
@@ -10418,7 +10418,7 @@
         </is>
       </c>
       <c r="AA19" s="12" t="n">
-        <v>24290</v>
+        <v>23200</v>
       </c>
       <c r="AB19" s="12" t="inlineStr">
         <is>
@@ -23848,7 +23848,7 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>SKLU1586238</t>
+          <t>SKLU2101727</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -23868,7 +23868,7 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>2120</t>
+          <t>1409</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
@@ -23914,7 +23914,7 @@
       </c>
       <c r="O15" s="12" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="P15" s="12" t="n"/>
@@ -23961,12 +23961,12 @@
       <c r="AC15" s="12" t="n"/>
       <c r="AD15" s="12" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="AE15" s="12" t="inlineStr">
         <is>
-          <t>0010</t>
+          <t>1710</t>
         </is>
       </c>
       <c r="AF15" s="12" t="inlineStr">
@@ -23987,7 +23987,7 @@
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>SKLU2101727</t>
+          <t>SKLU1553830</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -24007,7 +24007,7 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>1409</t>
+          <t>1243</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
@@ -24053,7 +24053,7 @@
       </c>
       <c r="O16" s="12" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="P16" s="12" t="n"/>
@@ -24105,7 +24105,7 @@
       </c>
       <c r="AE16" s="12" t="inlineStr">
         <is>
-          <t>1710</t>
+          <t>1610</t>
         </is>
       </c>
       <c r="AF16" s="12" t="inlineStr">
@@ -24126,7 +24126,7 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>SKLU2105770</t>
+          <t>SKLU1586238</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -24146,7 +24146,7 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>2305</t>
+          <t>2120</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
@@ -24192,7 +24192,7 @@
       </c>
       <c r="O17" s="12" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="P17" s="12" t="n"/>
@@ -24244,7 +24244,7 @@
       </c>
       <c r="AE17" s="12" t="inlineStr">
         <is>
-          <t>0210</t>
+          <t>0010</t>
         </is>
       </c>
       <c r="AF17" s="12" t="inlineStr">
@@ -24404,7 +24404,7 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>SKLU1553830</t>
+          <t>SKLU2105770</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -24424,7 +24424,7 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>1243</t>
+          <t>2305</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
@@ -24470,7 +24470,7 @@
       </c>
       <c r="O19" s="12" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="P19" s="12" t="n"/>
@@ -24517,12 +24517,12 @@
       <c r="AC19" s="12" t="n"/>
       <c r="AD19" s="12" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="AE19" s="12" t="inlineStr">
         <is>
-          <t>1610</t>
+          <t>0210</t>
         </is>
       </c>
       <c r="AF19" s="12" t="inlineStr">

</xml_diff>